<commit_message>
Refresh India AI repository after telecom/energy/materials agent final flush
Recompiled AI_Adoption_India_Repository.xlsx to fold in the finalized
F_telecom_energy_materials.jsonl records (de-duplicated by URL).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VTizj7RTVJtjNHzmVSnKMg
</commit_message>
<xml_diff>
--- a/stock-analysis/AI_Adoption_India_Repository.xlsx
+++ b/stock-analysis/AI_Adoption_India_Repository.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>352 unique sources · 100 companies · 11 sector groups (this pass).</t>
+          <t>352 unique sources · 100 companies · 10 sector groups (this pass).</t>
         </is>
       </c>
     </row>
@@ -5848,148 +5848,148 @@
     <row r="108" ht="44" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Energy &amp; Utilities</t>
+          <t>Energy, Power &amp; Utilities</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Petrochemicals</t>
+          <t>Power Transmission</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Reliance Industries</t>
+          <t>Adani Energy Solutions</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ADANIENSOL</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Grid/Energy optimization</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Reliance plans world's first fully autonomous refinery at Jamnagar</t>
+          <t>Adani Energy Solutions wins Rs 8,500 crore transmission project to power Vizag data centres and green energy hubs</t>
         </is>
       </c>
       <c r="G108" s="6" t="inlineStr">
         <is>
-          <t>ChemIndigest</t>
+          <t>Telangana Today</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr"/>
       <c r="I108" s="9" t="inlineStr">
         <is>
-          <t>Reliance plans to convert Jamnagar refinery into a fully AI-governed autonomous facility, per Anant Ambani at AGM.</t>
+          <t>Adani Energy Solutions won an Rs 8,500 crore transmission project to power AI infrastructure and data centres in Vizag.</t>
         </is>
       </c>
       <c r="J108" s="10" t="inlineStr">
         <is>
-          <t>https://chemindigest.com/reliance-plans-worlds-first-full...</t>
+          <t>https://telanganatoday.com/adani-energy-solutions-wins-rs...</t>
         </is>
       </c>
     </row>
     <row r="109" ht="44" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
         <is>
-          <t>Energy &amp; Utilities</t>
+          <t>Energy, Power &amp; Utilities</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Petrochemicals</t>
+          <t>Power Transmission</t>
         </is>
       </c>
       <c r="C109" s="12" t="inlineStr">
         <is>
-          <t>Reliance Industries</t>
+          <t>Adani Energy Solutions</t>
         </is>
       </c>
       <c r="D109" s="13" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ADANIENSOL</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Grid/Energy optimization</t>
         </is>
       </c>
       <c r="F109" s="14" t="inlineStr">
         <is>
-          <t>Reliance to turn Jamnagar complex into world's 1st fully autonomous refinery</t>
+          <t>Adani Energy Solutions Wins INR 8,500 Crore Transmission Project in Andhra Pradesh</t>
         </is>
       </c>
       <c r="G109" s="11" t="inlineStr">
         <is>
-          <t>Inshorts</t>
-        </is>
-      </c>
-      <c r="H109" s="13" t="inlineStr"/>
+          <t>SolarQuarter</t>
+        </is>
+      </c>
+      <c r="H109" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
       <c r="I109" s="14" t="inlineStr">
         <is>
-          <t>Reliance's Anant Ambani announced plans at the 49th AGM to build an AI-driven self-governing Jamnagar refinery.</t>
+          <t>New transmission project will deliver 4,500 MW to support green hydrogen and AI/hyperscale data centre demand.</t>
         </is>
       </c>
       <c r="J109" s="15" t="inlineStr">
         <is>
-          <t>https://inshorts.com/en/news/reliance-to-turn-jamnagar-co...</t>
+          <t>https://solarquarter.com/2026/07/24/adani-energy-solution...</t>
         </is>
       </c>
     </row>
     <row r="110" ht="44" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Energy &amp; Utilities</t>
+          <t>Energy, Power &amp; Utilities</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Petrochemicals</t>
+          <t>Power Generation</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>Reliance Industries</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Predictive maintenance</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Reliance AI Autonomous Refinery Jamnagar</t>
+          <t>India's Adani Power Selects Black &amp; Veatch to Optimize Thermal Power Assets, Reduce Operational Costs and Emissions</t>
         </is>
       </c>
       <c r="G110" s="6" t="inlineStr">
         <is>
-          <t>Channel I Am</t>
-        </is>
-      </c>
-      <c r="H110" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
+          <t>Black &amp; Veatch</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr"/>
       <c r="I110" s="9" t="inlineStr">
         <is>
-          <t>Reliance developed a proprietary AI feedstock optimisation tool to select efficient crude blends at Jamnagar.</t>
+          <t>Adani Power appointed Black &amp; Veatch to deploy predictive analytics software across 23 thermal units totaling ~12 GW.</t>
         </is>
       </c>
       <c r="J110" s="10" t="inlineStr">
         <is>
-          <t>https://en.channeliam.com/2026/06/22/reliance-ai-autonomo...</t>
+          <t>https://www.bv.com/en-US/news/indias-adani-power-selects-...</t>
         </is>
       </c>
     </row>
@@ -6001,43 +6001,43 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Power Transmission</t>
+          <t>Oil &amp; Gas Refining/Marketing</t>
         </is>
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>Adani Energy Solutions</t>
+          <t>Bharat Petroleum Corporation</t>
         </is>
       </c>
       <c r="D111" s="13" t="inlineStr">
         <is>
-          <t>ADANIENSOL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr">
         <is>
-          <t>Grid/Energy optimization</t>
+          <t>Churn/CX</t>
         </is>
       </c>
       <c r="F111" s="14" t="inlineStr">
         <is>
-          <t>Adani Energy Solutions wins Rs 8,500 crore transmission project to power Vizag data centres and green energy hubs</t>
+          <t>How BPCL is using Technology to accelerate Digital Transformation</t>
         </is>
       </c>
       <c r="G111" s="11" t="inlineStr">
         <is>
-          <t>Telangana Today</t>
+          <t>W.Media</t>
         </is>
       </c>
       <c r="H111" s="13" t="inlineStr"/>
       <c r="I111" s="14" t="inlineStr">
         <is>
-          <t>Adani Energy Solutions won an Rs 8,500 crore transmission project to power AI infrastructure and data centres in Vizag.</t>
+          <t>BPCL launched 'Urja', an AI/NLP virtual assistant trained on 600+ use cases for B2B and B2C customer queries.</t>
         </is>
       </c>
       <c r="J111" s="15" t="inlineStr">
         <is>
-          <t>https://telanganatoday.com/adani-energy-solutions-wins-rs...</t>
+          <t>https://w.media/how-bpcl-is-using-technology-to-accelerat...</t>
         </is>
       </c>
     </row>
@@ -6049,47 +6049,43 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Power Transmission</t>
+          <t>Oil &amp; Gas Refining/Marketing</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>Adani Energy Solutions</t>
+          <t>Bharat Petroleum Corporation</t>
         </is>
       </c>
       <c r="D112" s="8" t="inlineStr">
         <is>
-          <t>ADANIENSOL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t>Grid/Energy optimization</t>
+          <t>Churn/CX</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>Adani Energy Solutions Wins INR 8,500 Crore Transmission Project in Andhra Pradesh</t>
+          <t>BPCL partners with Microsoft to transform customer experience</t>
         </is>
       </c>
       <c r="G112" s="6" t="inlineStr">
         <is>
-          <t>SolarQuarter</t>
-        </is>
-      </c>
-      <c r="H112" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
+          <t>Technology Record</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr"/>
       <c r="I112" s="9" t="inlineStr">
         <is>
-          <t>New transmission project will deliver 4,500 MW to support green hydrogen and AI/hyperscale data centre demand.</t>
+          <t>BPCL partnered with Microsoft to use cloud and AI to drive digital transformation and customer experience.</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
         <is>
-          <t>https://solarquarter.com/2026/07/24/adani-energy-solution...</t>
+          <t>https://www.technologyrecord.com/article/bpcl-partners-wi...</t>
         </is>
       </c>
     </row>
@@ -6101,43 +6097,43 @@
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Power Generation</t>
+          <t>Oil &amp; Gas Refining/Marketing</t>
         </is>
       </c>
       <c r="C113" s="12" t="inlineStr">
         <is>
-          <t>Adani Power</t>
+          <t>Bharat Petroleum Corporation</t>
         </is>
       </c>
       <c r="D113" s="13" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="E113" s="13" t="inlineStr">
         <is>
-          <t>Predictive maintenance</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F113" s="14" t="inlineStr">
         <is>
-          <t>India's Adani Power Selects Black &amp; Veatch to Optimize Thermal Power Assets, Reduce Operational Costs and Emissions</t>
+          <t>Enhancing the Efficiency of Refining Processes: A Desktop Solution for Predicting FCC Yield Profiles</t>
         </is>
       </c>
       <c r="G113" s="11" t="inlineStr">
         <is>
-          <t>Black &amp; Veatch</t>
+          <t>OnePetro (SPE ADIP)</t>
         </is>
       </c>
       <c r="H113" s="13" t="inlineStr"/>
       <c r="I113" s="14" t="inlineStr">
         <is>
-          <t>Adani Power appointed Black &amp; Veatch to deploy predictive analytics software across 23 thermal units totaling ~12 GW.</t>
+          <t>BPCL R&amp;D developed a proprietary AI-based Yield Prediction model to streamline FCC catalyst testing and selection.</t>
         </is>
       </c>
       <c r="J113" s="15" t="inlineStr">
         <is>
-          <t>https://www.bv.com/en-US/news/indias-adani-power-selects-...</t>
+          <t>https://onepetro.org/SPEADIP/proceedings-abstract/24ADIP/...</t>
         </is>
       </c>
     </row>
@@ -6164,28 +6160,32 @@
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>Churn/CX</t>
+          <t>Demand forecasting</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>How BPCL is using Technology to accelerate Digital Transformation</t>
+          <t>Accenture helps to digitally transform BPCL's sales and distribution network using AI and Machine Learning</t>
         </is>
       </c>
       <c r="G114" s="6" t="inlineStr">
         <is>
-          <t>W.Media</t>
-        </is>
-      </c>
-      <c r="H114" s="8" t="inlineStr"/>
+          <t>Accenture Newsroom</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="I114" s="9" t="inlineStr">
         <is>
-          <t>BPCL launched 'Urja', an AI/NLP virtual assistant trained on 600+ use cases for B2B and B2C customer queries.</t>
+          <t>BPCL built AI/cloud platform IRIS integrating real-time data from 18,000+ retail outlets and 25,000 tank trucks.</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
         <is>
-          <t>https://w.media/how-bpcl-is-using-technology-to-accelerat...</t>
+          <t>https://newsroom.accenture.com/news/2021/bharat-petroleum...</t>
         </is>
       </c>
     </row>
@@ -6197,43 +6197,43 @@
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Marketing</t>
+          <t>Coal Mining</t>
         </is>
       </c>
       <c r="C115" s="12" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation</t>
+          <t>Coal India</t>
         </is>
       </c>
       <c r="D115" s="13" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="E115" s="13" t="inlineStr">
         <is>
-          <t>Churn/CX</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F115" s="14" t="inlineStr">
         <is>
-          <t>BPCL partners with Microsoft to transform customer experience</t>
+          <t>Coal India Partners with ISRO's NRSC to Develop AI-Powered Satellite Dashboard for Smart Mine Monitoring</t>
         </is>
       </c>
       <c r="G115" s="11" t="inlineStr">
         <is>
-          <t>Technology Record</t>
+          <t>Indian Masterminds</t>
         </is>
       </c>
       <c r="H115" s="13" t="inlineStr"/>
       <c r="I115" s="14" t="inlineStr">
         <is>
-          <t>BPCL partnered with Microsoft to use cloud and AI to drive digital transformation and customer experience.</t>
+          <t>AI/ML and deep learning integrated with ISRO satellite data will track mine closure, land reclamation and illegal mining.</t>
         </is>
       </c>
       <c r="J115" s="15" t="inlineStr">
         <is>
-          <t>https://www.technologyrecord.com/article/bpcl-partners-wi...</t>
+          <t>https://indianmasterminds.com/news/coal-india-isro-nrsc-a...</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6245,17 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Marketing</t>
+          <t>Coal Mining</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation</t>
+          <t>Coal India</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -6265,23 +6265,27 @@
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Enhancing the Efficiency of Refining Processes: A Desktop Solution for Predicting FCC Yield Profiles</t>
+          <t>Coal India Partners with ISRO's NRSC to Build AI-Based Satellite Monitoring System for Mines</t>
         </is>
       </c>
       <c r="G116" s="6" t="inlineStr">
         <is>
-          <t>OnePetro (SPE ADIP)</t>
-        </is>
-      </c>
-      <c r="H116" s="8" t="inlineStr"/>
+          <t>Elets eGov</t>
+        </is>
+      </c>
+      <c r="H116" s="8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
       <c r="I116" s="9" t="inlineStr">
         <is>
-          <t>BPCL R&amp;D developed a proprietary AI-based Yield Prediction model to streamline FCC catalyst testing and selection.</t>
+          <t>Coal India signed an MoU with ISRO's NRSC for an AI-powered satellite geospatial dashboard monitoring mine operations.</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
         <is>
-          <t>https://onepetro.org/SPEADIP/proceedings-abstract/24ADIP/...</t>
+          <t>https://egov.eletsonline.com/2026/07/coal-india-partners-...</t>
         </is>
       </c>
     </row>
@@ -6293,47 +6297,43 @@
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining/Marketing</t>
+          <t>Natural Gas Transmission</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation</t>
+          <t>GAIL (India)</t>
         </is>
       </c>
       <c r="D117" s="13" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="E117" s="13" t="inlineStr">
         <is>
-          <t>Demand forecasting</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F117" s="14" t="inlineStr">
         <is>
-          <t>Accenture helps to digitally transform BPCL's sales and distribution network using AI and Machine Learning</t>
+          <t>GAIL Bets Big On Pipelines And AI To Power India's Gas Push</t>
         </is>
       </c>
       <c r="G117" s="11" t="inlineStr">
         <is>
-          <t>Accenture Newsroom</t>
-        </is>
-      </c>
-      <c r="H117" s="13" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
+          <t>The Core</t>
+        </is>
+      </c>
+      <c r="H117" s="13" t="inlineStr"/>
       <c r="I117" s="14" t="inlineStr">
         <is>
-          <t>BPCL built AI/cloud platform IRIS integrating real-time data from 18,000+ retail outlets and 25,000 tank trucks.</t>
+          <t>GAIL is expanding its gas pipeline network while investing in AI capability building for operational efficiency.</t>
         </is>
       </c>
       <c r="J117" s="15" t="inlineStr">
         <is>
-          <t>https://newsroom.accenture.com/news/2021/bharat-petroleum...</t>
+          <t>https://www.thecore.in/business/gail-ai-pipelines-india-e...</t>
         </is>
       </c>
     </row>
@@ -6345,17 +6345,17 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>Coal Mining</t>
+          <t>Natural Gas Transmission</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>Coal India</t>
+          <t>GAIL (India)</t>
         </is>
       </c>
       <c r="D118" s="8" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -6365,23 +6365,23 @@
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Coal India Partners with ISRO's NRSC to Develop AI-Powered Satellite Dashboard for Smart Mine Monitoring</t>
+          <t>GAIL AI Tarang - Artificial Intelligence Literacy and Capacity Building initiative</t>
         </is>
       </c>
       <c r="G118" s="6" t="inlineStr">
         <is>
-          <t>Indian Masterminds</t>
+          <t>GAIL India (X/Twitter)</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr"/>
       <c r="I118" s="9" t="inlineStr">
         <is>
-          <t>AI/ML and deep learning integrated with ISRO satellite data will track mine closure, land reclamation and illegal mining.</t>
+          <t>GAIL launched 'AI Tarang', training over 3,700 of its 5,000 employees in AI fundamentals for the organization.</t>
         </is>
       </c>
       <c r="J118" s="10" t="inlineStr">
         <is>
-          <t>https://indianmasterminds.com/news/coal-india-isro-nrsc-a...</t>
+          <t>https://x.com/gailindia/status/1958438772988686675</t>
         </is>
       </c>
     </row>
@@ -6393,17 +6393,17 @@
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Coal Mining</t>
+          <t>Natural Gas Transmission</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>Coal India</t>
+          <t>GAIL (India)</t>
         </is>
       </c>
       <c r="D119" s="13" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="E119" s="13" t="inlineStr">
@@ -6413,27 +6413,23 @@
       </c>
       <c r="F119" s="14" t="inlineStr">
         <is>
-          <t>Coal India Partners with ISRO's NRSC to Build AI-Based Satellite Monitoring System for Mines</t>
+          <t>GAIL India company profile</t>
         </is>
       </c>
       <c r="G119" s="11" t="inlineStr">
         <is>
-          <t>Elets eGov</t>
-        </is>
-      </c>
-      <c r="H119" s="13" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
+          <t>AI Magazine</t>
+        </is>
+      </c>
+      <c r="H119" s="13" t="inlineStr"/>
       <c r="I119" s="14" t="inlineStr">
         <is>
-          <t>Coal India signed an MoU with ISRO's NRSC for an AI-powered satellite geospatial dashboard monitoring mine operations.</t>
+          <t>Company profile covering GAIL India's role and technology adoption within the natural gas value chain.</t>
         </is>
       </c>
       <c r="J119" s="15" t="inlineStr">
         <is>
-          <t>https://egov.eletsonline.com/2026/07/coal-india-partners-...</t>
+          <t>https://aimagazine.com/company/gail-india</t>
         </is>
       </c>
     </row>
@@ -6445,19 +6441,15 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Natural Gas Transmission</t>
+          <t>Oil &amp; Gas Refining</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>GAIL (India)</t>
-        </is>
-      </c>
-      <c r="D120" s="8" t="inlineStr">
-        <is>
-          <t>GAIL</t>
-        </is>
-      </c>
+          <t>Indian refining sector (IOC/BPCL/HPCL)</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr"/>
       <c r="E120" s="8" t="inlineStr">
         <is>
           <t>Process/Yield</t>
@@ -6465,23 +6457,23 @@
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>GAIL Bets Big On Pipelines And AI To Power India's Gas Push</t>
+          <t>Oil firms are embracing digital tech to drive operational efficiency</t>
         </is>
       </c>
       <c r="G120" s="6" t="inlineStr">
         <is>
-          <t>The Core</t>
+          <t>Business Standard</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr"/>
       <c r="I120" s="9" t="inlineStr">
         <is>
-          <t>GAIL is expanding its gas pipeline network while investing in AI capability building for operational efficiency.</t>
+          <t>Indian refiners adopting digital technologies including AI-based corrosion management, predictive maintenance and drone inspection.</t>
         </is>
       </c>
       <c r="J120" s="10" t="inlineStr">
         <is>
-          <t>https://www.thecore.in/business/gail-ai-pipelines-india-e...</t>
+          <t>https://www.business-standard.com/amp/article/companies/o...</t>
         </is>
       </c>
     </row>
@@ -6493,43 +6485,47 @@
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>Natural Gas Transmission</t>
+          <t>Power Generation</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>GAIL (India)</t>
+          <t>JSW Energy</t>
         </is>
       </c>
       <c r="D121" s="13" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>JSWENERGY</t>
         </is>
       </c>
       <c r="E121" s="13" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Predictive maintenance</t>
         </is>
       </c>
       <c r="F121" s="14" t="inlineStr">
         <is>
-          <t>GAIL AI Tarang - Artificial Intelligence Literacy and Capacity Building initiative</t>
+          <t>JSW Energy Investment Guide 2025 - Business Model, Financial Performance &amp; Future Growth Potential</t>
         </is>
       </c>
       <c r="G121" s="11" t="inlineStr">
         <is>
-          <t>GAIL India (X/Twitter)</t>
-        </is>
-      </c>
-      <c r="H121" s="13" t="inlineStr"/>
+          <t>StocksCaseStudy</t>
+        </is>
+      </c>
+      <c r="H121" s="13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="I121" s="14" t="inlineStr">
         <is>
-          <t>GAIL launched 'AI Tarang', training over 3,700 of its 5,000 employees in AI fundamentals for the organization.</t>
+          <t>JSW Energy uses IoT to forecast power generation needs in 15-minute cycles and plans AI-based predictive maintenance.</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr">
         <is>
-          <t>https://x.com/gailindia/status/1958438772988686675</t>
+          <t>https://stockscasestudy.com/jsw-energy-investment-guide-2...</t>
         </is>
       </c>
     </row>
@@ -6541,43 +6537,43 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>Natural Gas Transmission</t>
+          <t>Power Generation</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>GAIL (India)</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="D122" s="8" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Predictive maintenance</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>GAIL India company profile</t>
+          <t>Toshiba to set up AI monitoring at 165 Indian power plants</t>
         </is>
       </c>
       <c r="G122" s="6" t="inlineStr">
         <is>
-          <t>AI Magazine</t>
+          <t>Manufacturing Today India</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr"/>
       <c r="I122" s="9" t="inlineStr">
         <is>
-          <t>Company profile covering GAIL India's role and technology adoption within the natural gas value chain.</t>
+          <t>NTPC's first plant-wide AI monitoring deployment will analyze sensor data for early abnormality detection.</t>
         </is>
       </c>
       <c r="J122" s="10" t="inlineStr">
         <is>
-          <t>https://aimagazine.com/company/gail-india</t>
+          <t>https://www.manufacturingtodayindia.com/toshiba-to-set-up...</t>
         </is>
       </c>
     </row>
@@ -6589,39 +6585,43 @@
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Refining</t>
+          <t>Power Generation</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>Indian refining sector (IOC/BPCL/HPCL)</t>
-        </is>
-      </c>
-      <c r="D123" s="13" t="inlineStr"/>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D123" s="13" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
       <c r="E123" s="13" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Predictive maintenance</t>
         </is>
       </c>
       <c r="F123" s="14" t="inlineStr">
         <is>
-          <t>Oil firms are embracing digital tech to drive operational efficiency</t>
+          <t>Toshiba to deploy EtaPRO AI-driven monitoring system at 165 power plants in India</t>
         </is>
       </c>
       <c r="G123" s="11" t="inlineStr">
         <is>
-          <t>Business Standard</t>
+          <t>EPR Magazine</t>
         </is>
       </c>
       <c r="H123" s="13" t="inlineStr"/>
       <c r="I123" s="14" t="inlineStr">
         <is>
-          <t>Indian refiners adopting digital technologies including AI-based corrosion management, predictive maintenance and drone inspection.</t>
+          <t>AI system will perform root cause analysis and automate maintenance processes across NTPC's power fleet.</t>
         </is>
       </c>
       <c r="J123" s="15" t="inlineStr">
         <is>
-          <t>https://www.business-standard.com/amp/article/companies/o...</t>
+          <t>https://www.eprmagazine.com/power-brand/toshiba-to-deploy...</t>
         </is>
       </c>
     </row>
@@ -6638,12 +6638,12 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>JSW Energy</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="D124" s="8" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
@@ -6653,27 +6653,23 @@
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>JSW Energy Investment Guide 2025 - Business Model, Financial Performance &amp; Future Growth Potential</t>
+          <t>Toshiba to Deploy EtaPRO AI-Driven Monitoring System at 165 Power Plants in India</t>
         </is>
       </c>
       <c r="G124" s="6" t="inlineStr">
         <is>
-          <t>StocksCaseStudy</t>
-        </is>
-      </c>
-      <c r="H124" s="8" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+          <t>Toshiba UK Newsroom</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="inlineStr"/>
       <c r="I124" s="9" t="inlineStr">
         <is>
-          <t>JSW Energy uses IoT to forecast power generation needs in 15-minute cycles and plans AI-based predictive maintenance.</t>
+          <t>Centralized AI monitoring system for NTPC begins operations in 2027 covering thermal and renewable generation.</t>
         </is>
       </c>
       <c r="J124" s="10" t="inlineStr">
         <is>
-          <t>https://stockscasestudy.com/jsw-energy-investment-guide-2...</t>
+          <t>https://www.toshiba.co.uk/newsroom/toshiba-to-deploy-etap...</t>
         </is>
       </c>
     </row>
@@ -6705,23 +6701,23 @@
       </c>
       <c r="F125" s="14" t="inlineStr">
         <is>
-          <t>Toshiba to set up AI monitoring at 165 Indian power plants</t>
+          <t>EtaPRO - AI-Driven Monitoring and Diagnostics Solution to Be Deployed Across Up to 165 Power Plants in India</t>
         </is>
       </c>
       <c r="G125" s="11" t="inlineStr">
         <is>
-          <t>Manufacturing Today India</t>
+          <t>EtaPRO</t>
         </is>
       </c>
       <c r="H125" s="13" t="inlineStr"/>
       <c r="I125" s="14" t="inlineStr">
         <is>
-          <t>NTPC's first plant-wide AI monitoring deployment will analyze sensor data for early abnormality detection.</t>
+          <t>EtaPRO's global predictive diagnostics platform, already covering 763 GW worldwide, will now serve NTPC's fleet.</t>
         </is>
       </c>
       <c r="J125" s="15" t="inlineStr">
         <is>
-          <t>https://www.manufacturingtodayindia.com/toshiba-to-set-up...</t>
+          <t>https://etapro.com/news-events/etapro-ai-driven-monitorin...</t>
         </is>
       </c>
     </row>
@@ -6753,23 +6749,27 @@
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Toshiba to deploy EtaPRO AI-driven monitoring system at 165 power plants in India</t>
+          <t>Toshiba to Deploy EtaPRO(TM) AI-Driven Monitoring System at 165 Power Plants in India</t>
         </is>
       </c>
       <c r="G126" s="6" t="inlineStr">
         <is>
-          <t>EPR Magazine</t>
-        </is>
-      </c>
-      <c r="H126" s="8" t="inlineStr"/>
+          <t>Toshiba Energy Systems &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="inlineStr">
+        <is>
+          <t>2025-10-09</t>
+        </is>
+      </c>
       <c r="I126" s="9" t="inlineStr">
         <is>
-          <t>AI system will perform root cause analysis and automate maintenance processes across NTPC's power fleet.</t>
+          <t>Toshiba JSW Power Systems will deploy AI-based centralized monitoring across 165 NTPC thermal and renewable plants.</t>
         </is>
       </c>
       <c r="J126" s="10" t="inlineStr">
         <is>
-          <t>https://www.eprmagazine.com/power-brand/toshiba-to-deploy...</t>
+          <t>https://www.global.toshiba/ww/news/energy/2025/10/news-20...</t>
         </is>
       </c>
     </row>
@@ -6781,43 +6781,43 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>Power Generation</t>
+          <t>Oil &amp; Gas Exploration</t>
         </is>
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>Oil and Natural Gas Corporation</t>
         </is>
       </c>
       <c r="D127" s="13" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="E127" s="13" t="inlineStr">
         <is>
-          <t>Predictive maintenance</t>
+          <t>Exploration analytics</t>
         </is>
       </c>
       <c r="F127" s="14" t="inlineStr">
         <is>
-          <t>Toshiba to Deploy EtaPRO AI-Driven Monitoring System at 165 Power Plants in India</t>
+          <t>ONGC Turns To AI-Led Drilling To Crack Deepwater Exploration Challenge</t>
         </is>
       </c>
       <c r="G127" s="11" t="inlineStr">
         <is>
-          <t>Toshiba UK Newsroom</t>
+          <t>The Core</t>
         </is>
       </c>
       <c r="H127" s="13" t="inlineStr"/>
       <c r="I127" s="14" t="inlineStr">
         <is>
-          <t>Centralized AI monitoring system for NTPC begins operations in 2027 covering thermal and renewable generation.</t>
+          <t>ONGC's AI-driven well location drilling achieved 98.5% accuracy, aiding deepwater exploration and reservoir characterization.</t>
         </is>
       </c>
       <c r="J127" s="15" t="inlineStr">
         <is>
-          <t>https://www.toshiba.co.uk/newsroom/toshiba-to-deploy-etap...</t>
+          <t>https://www.thecore.in/economy/ongc-turns-to-ai-led-drill...</t>
         </is>
       </c>
     </row>
@@ -6829,43 +6829,43 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>Power Generation</t>
+          <t>Oil &amp; Gas Exploration</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>Oil and Natural Gas Corporation</t>
         </is>
       </c>
       <c r="D128" s="8" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
         <is>
-          <t>Predictive maintenance</t>
+          <t>Exploration analytics</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>EtaPRO - AI-Driven Monitoring and Diagnostics Solution to Be Deployed Across Up to 165 Power Plants in India</t>
+          <t>Navigating depths: ONGC's deepwater exploration challenges &amp; innovations</t>
         </is>
       </c>
       <c r="G128" s="6" t="inlineStr">
         <is>
-          <t>EtaPRO</t>
+          <t>Millennium Post</t>
         </is>
       </c>
       <c r="H128" s="8" t="inlineStr"/>
       <c r="I128" s="9" t="inlineStr">
         <is>
-          <t>EtaPRO's global predictive diagnostics platform, already covering 763 GW worldwide, will now serve NTPC's fleet.</t>
+          <t>ONGC leverages AI and digital centralization to improve exploration success in high-risk deepwater fields.</t>
         </is>
       </c>
       <c r="J128" s="10" t="inlineStr">
         <is>
-          <t>https://etapro.com/news-events/etapro-ai-driven-monitorin...</t>
+          <t>https://www.millenniumpost.in/business/navigating-depths-...</t>
         </is>
       </c>
     </row>
@@ -6877,47 +6877,43 @@
       </c>
       <c r="B129" s="11" t="inlineStr">
         <is>
-          <t>Power Generation</t>
+          <t>Oil &amp; Gas Exploration</t>
         </is>
       </c>
       <c r="C129" s="12" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>Oil and Natural Gas Corporation</t>
         </is>
       </c>
       <c r="D129" s="13" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="E129" s="13" t="inlineStr">
         <is>
-          <t>Predictive maintenance</t>
+          <t>Exploration analytics</t>
         </is>
       </c>
       <c r="F129" s="14" t="inlineStr">
         <is>
-          <t>Toshiba to Deploy EtaPRO(TM) AI-Driven Monitoring System at 165 Power Plants in India</t>
+          <t>Case Study: An Agentic AI Framework for Large-Scale Well Modeling of Offshore Field Developments</t>
         </is>
       </c>
       <c r="G129" s="11" t="inlineStr">
         <is>
-          <t>Toshiba Energy Systems &amp; Solutions</t>
-        </is>
-      </c>
-      <c r="H129" s="13" t="inlineStr">
-        <is>
-          <t>2025-10-09</t>
-        </is>
-      </c>
+          <t>JPT (SPE)</t>
+        </is>
+      </c>
+      <c r="H129" s="13" t="inlineStr"/>
       <c r="I129" s="14" t="inlineStr">
         <is>
-          <t>Toshiba JSW Power Systems will deploy AI-based centralized monitoring across 165 NTPC thermal and renewable plants.</t>
+          <t>Supervised agentic AI automation scaled well modeling across hundreds of ONGC offshore wells, saving 1,000+ engineering hours.</t>
         </is>
       </c>
       <c r="J129" s="15" t="inlineStr">
         <is>
-          <t>https://www.global.toshiba/ww/news/energy/2025/10/news-20...</t>
+          <t>https://jpt.spe.org/case-study-an-agentic-ai-framework-fo...</t>
         </is>
       </c>
     </row>
@@ -6949,23 +6945,23 @@
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>ONGC Turns To AI-Led Drilling To Crack Deepwater Exploration Challenge</t>
+          <t>ONGC Leads AI Revolution in Oil and Gas Optimization</t>
         </is>
       </c>
       <c r="G130" s="6" t="inlineStr">
         <is>
-          <t>The Core</t>
+          <t>Visive.ai</t>
         </is>
       </c>
       <c r="H130" s="8" t="inlineStr"/>
       <c r="I130" s="9" t="inlineStr">
         <is>
-          <t>ONGC's AI-driven well location drilling achieved 98.5% accuracy, aiding deepwater exploration and reservoir characterization.</t>
+          <t>Coverage of ONGC's AI investment in reservoir management, drilling optimization and remote autonomous operations.</t>
         </is>
       </c>
       <c r="J130" s="10" t="inlineStr">
         <is>
-          <t>https://www.thecore.in/economy/ongc-turns-to-ai-led-drill...</t>
+          <t>https://www.visive.ai/news/ongc-leads-ai-revolution-in-oi...</t>
         </is>
       </c>
     </row>
@@ -6997,23 +6993,27 @@
       </c>
       <c r="F131" s="14" t="inlineStr">
         <is>
-          <t>Navigating depths: ONGC's deepwater exploration challenges &amp; innovations</t>
+          <t>ONGC Introduces AI-Driven Well Information System to Enhance Drilling Efficiency</t>
         </is>
       </c>
       <c r="G131" s="11" t="inlineStr">
         <is>
-          <t>Millennium Post</t>
-        </is>
-      </c>
-      <c r="H131" s="13" t="inlineStr"/>
+          <t>APAC News Network</t>
+        </is>
+      </c>
+      <c r="H131" s="13" t="inlineStr">
+        <is>
+          <t>2024-12-20</t>
+        </is>
+      </c>
       <c r="I131" s="14" t="inlineStr">
         <is>
-          <t>ONGC leverages AI and digital centralization to improve exploration success in high-risk deepwater fields.</t>
+          <t>ONGC unveiled a generative-AI-powered Well Information System for real-time monitoring and centralized drilling management.</t>
         </is>
       </c>
       <c r="J131" s="15" t="inlineStr">
         <is>
-          <t>https://www.millenniumpost.in/business/navigating-depths-...</t>
+          <t>https://apacnewsnetwork.com/2024/12/ongc-introduces-ai-dr...</t>
         </is>
       </c>
     </row>
@@ -7025,43 +7025,43 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Exploration</t>
+          <t>Power Transmission</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas Corporation</t>
+          <t>Power Grid Corporation of India</t>
         </is>
       </c>
       <c r="D132" s="8" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>Exploration analytics</t>
+          <t>Grid/Energy optimization</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>Case Study: An Agentic AI Framework for Large-Scale Well Modeling of Offshore Field Developments</t>
+          <t>India to Embed AI in National Power Grid to Cut Maintenance Costs, Energy Losses</t>
         </is>
       </c>
       <c r="G132" s="6" t="inlineStr">
         <is>
-          <t>JPT (SPE)</t>
+          <t>Outlook Business</t>
         </is>
       </c>
       <c r="H132" s="8" t="inlineStr"/>
       <c r="I132" s="9" t="inlineStr">
         <is>
-          <t>Supervised agentic AI automation scaled well modeling across hundreds of ONGC offshore wells, saving 1,000+ engineering hours.</t>
+          <t>India plans AI deployment in the national grid for real-time fault prediction and market surveillance.</t>
         </is>
       </c>
       <c r="J132" s="10" t="inlineStr">
         <is>
-          <t>https://jpt.spe.org/case-study-an-agentic-ai-framework-fo...</t>
+          <t>https://www.outlookbusiness.com/industry/india-ai-power-g...</t>
         </is>
       </c>
     </row>
@@ -7073,43 +7073,43 @@
       </c>
       <c r="B133" s="11" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Exploration</t>
+          <t>Power Transmission</t>
         </is>
       </c>
       <c r="C133" s="12" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas Corporation</t>
+          <t>Power Grid Corporation of India</t>
         </is>
       </c>
       <c r="D133" s="13" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="E133" s="13" t="inlineStr">
         <is>
-          <t>Exploration analytics</t>
+          <t>Grid/Energy optimization</t>
         </is>
       </c>
       <c r="F133" s="14" t="inlineStr">
         <is>
-          <t>ONGC Leads AI Revolution in Oil and Gas Optimization</t>
+          <t>Optimizing India's Electricity Grid for Renewables Using AI and Machine Learning Applications</t>
         </is>
       </c>
       <c r="G133" s="11" t="inlineStr">
         <is>
-          <t>Visive.ai</t>
+          <t>CSIS</t>
         </is>
       </c>
       <c r="H133" s="13" t="inlineStr"/>
       <c r="I133" s="14" t="inlineStr">
         <is>
-          <t>Coverage of ONGC's AI investment in reservoir management, drilling optimization and remote autonomous operations.</t>
+          <t>CSIS analysis of AI/ML applications for India's grid including demand forecasting and renewable integration.</t>
         </is>
       </c>
       <c r="J133" s="15" t="inlineStr">
         <is>
-          <t>https://www.visive.ai/news/ongc-leads-ai-revolution-in-oi...</t>
+          <t>https://www.csis.org/analysis/optimizing-indias-electrici...</t>
         </is>
       </c>
     </row>
@@ -7121,47 +7121,43 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Exploration</t>
+          <t>Oil &amp; Gas Refining/Petrochemicals</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas Corporation</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="D134" s="8" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>Exploration analytics</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>ONGC Introduces AI-Driven Well Information System to Enhance Drilling Efficiency</t>
+          <t>Reliance plans world's first fully autonomous refinery at Jamnagar</t>
         </is>
       </c>
       <c r="G134" s="6" t="inlineStr">
         <is>
-          <t>APAC News Network</t>
-        </is>
-      </c>
-      <c r="H134" s="8" t="inlineStr">
-        <is>
-          <t>2024-12-20</t>
-        </is>
-      </c>
+          <t>ChemIndigest</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="inlineStr"/>
       <c r="I134" s="9" t="inlineStr">
         <is>
-          <t>ONGC unveiled a generative-AI-powered Well Information System for real-time monitoring and centralized drilling management.</t>
+          <t>Reliance plans to convert Jamnagar refinery into a fully AI-governed autonomous facility, per Anant Ambani at AGM.</t>
         </is>
       </c>
       <c r="J134" s="10" t="inlineStr">
         <is>
-          <t>https://apacnewsnetwork.com/2024/12/ongc-introduces-ai-dr...</t>
+          <t>https://chemindigest.com/reliance-plans-worlds-first-full...</t>
         </is>
       </c>
     </row>
@@ -7173,43 +7169,43 @@
       </c>
       <c r="B135" s="11" t="inlineStr">
         <is>
-          <t>Power Transmission</t>
+          <t>Oil &amp; Gas Refining/Petrochemicals</t>
         </is>
       </c>
       <c r="C135" s="12" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="D135" s="13" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="E135" s="13" t="inlineStr">
         <is>
-          <t>Grid/Energy optimization</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F135" s="14" t="inlineStr">
         <is>
-          <t>India to Embed AI in National Power Grid to Cut Maintenance Costs, Energy Losses</t>
+          <t>Reliance to turn Jamnagar complex into world's 1st fully autonomous refinery</t>
         </is>
       </c>
       <c r="G135" s="11" t="inlineStr">
         <is>
-          <t>Outlook Business</t>
+          <t>Inshorts</t>
         </is>
       </c>
       <c r="H135" s="13" t="inlineStr"/>
       <c r="I135" s="14" t="inlineStr">
         <is>
-          <t>India plans AI deployment in the national grid for real-time fault prediction and market surveillance.</t>
+          <t>Reliance's Anant Ambani announced plans at the 49th AGM to build an AI-driven self-governing Jamnagar refinery.</t>
         </is>
       </c>
       <c r="J135" s="15" t="inlineStr">
         <is>
-          <t>https://www.outlookbusiness.com/industry/india-ai-power-g...</t>
+          <t>https://inshorts.com/en/news/reliance-to-turn-jamnagar-co...</t>
         </is>
       </c>
     </row>
@@ -7221,43 +7217,47 @@
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>Power Transmission</t>
+          <t>Oil &amp; Gas Refining/Petrochemicals</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India</t>
+          <t>Reliance Industries</t>
         </is>
       </c>
       <c r="D136" s="8" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
         <is>
-          <t>Grid/Energy optimization</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>Optimizing India's Electricity Grid for Renewables Using AI and Machine Learning Applications</t>
+          <t>Reliance AI Autonomous Refinery Jamnagar</t>
         </is>
       </c>
       <c r="G136" s="6" t="inlineStr">
         <is>
-          <t>CSIS</t>
-        </is>
-      </c>
-      <c r="H136" s="8" t="inlineStr"/>
+          <t>Channel I Am</t>
+        </is>
+      </c>
+      <c r="H136" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="I136" s="9" t="inlineStr">
         <is>
-          <t>CSIS analysis of AI/ML applications for India's grid including demand forecasting and renewable integration.</t>
+          <t>Reliance developed a proprietary AI feedstock optimisation tool to select efficient crude blends at Jamnagar.</t>
         </is>
       </c>
       <c r="J136" s="10" t="inlineStr">
         <is>
-          <t>https://www.csis.org/analysis/optimizing-indias-electrici...</t>
+          <t>https://en.channeliam.com/2026/06/22/reliance-ai-autonomo...</t>
         </is>
       </c>
     </row>
@@ -15658,38 +15658,38 @@
       </c>
       <c r="C309" s="12" t="inlineStr">
         <is>
-          <t>Tata Steel</t>
+          <t>Steel Authority of India (SAIL)</t>
         </is>
       </c>
       <c r="D309" s="13" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SAIL</t>
         </is>
       </c>
       <c r="E309" s="13" t="inlineStr">
         <is>
-          <t>Digital twin</t>
+          <t>Process/Yield</t>
         </is>
       </c>
       <c r="F309" s="14" t="inlineStr">
         <is>
-          <t>How Digital Twin is a Game Changer for Tata Steel Nederland to Achieve Their Targets</t>
+          <t>How AI Is Reforging India's Steel Industry</t>
         </is>
       </c>
       <c r="G309" s="11" t="inlineStr">
         <is>
-          <t>Ansys</t>
+          <t>ARC Advisory Group</t>
         </is>
       </c>
       <c r="H309" s="13" t="inlineStr"/>
       <c r="I309" s="14" t="inlineStr">
         <is>
-          <t>Tata Steel's Netherlands operations use Ansys digital twin simulation to optimize plant performance and targets.</t>
+          <t>SAIL cited among major Indian steel players implementing AI-driven production monitoring and predictive maintenance.</t>
         </is>
       </c>
       <c r="J309" s="15" t="inlineStr">
         <is>
-          <t>https://www.ansys.com/webinars/how-digital-twin-is-a-game...</t>
+          <t>https://www.arcweb.com/blog/how-ai-reforging-indias-steel...</t>
         </is>
       </c>
     </row>
@@ -15721,23 +15721,23 @@
       </c>
       <c r="F310" s="9" t="inlineStr">
         <is>
-          <t>How Tata Steel has Transformed Plant And Mines With Digital Twins</t>
+          <t>How Digital Twin is a Game Changer for Tata Steel Nederland to Achieve Their Targets</t>
         </is>
       </c>
       <c r="G310" s="6" t="inlineStr">
         <is>
-          <t>Financial Express (Futech)</t>
+          <t>Ansys</t>
         </is>
       </c>
       <c r="H310" s="8" t="inlineStr"/>
       <c r="I310" s="9" t="inlineStr">
         <is>
-          <t>Tata Steel built digital twins of mines and manufacturing plants enabling remote monitoring and simulation.</t>
+          <t>Tata Steel's Netherlands operations use Ansys digital twin simulation to optimize plant performance and targets.</t>
         </is>
       </c>
       <c r="J310" s="10" t="inlineStr">
         <is>
-          <t>https://futech.financialexpressb2b.com/features/how-tata-...</t>
+          <t>https://www.ansys.com/webinars/how-digital-twin-is-a-game...</t>
         </is>
       </c>
     </row>
@@ -15769,23 +15769,23 @@
       </c>
       <c r="F311" s="14" t="inlineStr">
         <is>
-          <t>Tata Steel Digital Story</t>
+          <t>How Tata Steel has Transformed Plant And Mines With Digital Twins</t>
         </is>
       </c>
       <c r="G311" s="11" t="inlineStr">
         <is>
-          <t>IFQM</t>
+          <t>Financial Express (Futech)</t>
         </is>
       </c>
       <c r="H311" s="13" t="inlineStr"/>
       <c r="I311" s="14" t="inlineStr">
         <is>
-          <t>Case study documenting Tata Steel's digital transformation journey including AI and digital twin deployment.</t>
+          <t>Tata Steel built digital twins of mines and manufacturing plants enabling remote monitoring and simulation.</t>
         </is>
       </c>
       <c r="J311" s="15" t="inlineStr">
         <is>
-          <t>https://ifqm.org.in/product/tata-steel-digital-story/</t>
+          <t>https://futech.financialexpressb2b.com/features/how-tata-...</t>
         </is>
       </c>
     </row>
@@ -15817,23 +15817,23 @@
       </c>
       <c r="F312" s="9" t="inlineStr">
         <is>
-          <t>How Tata Steel has Transformed Plant And Mines With Digital Twins</t>
+          <t>Tata Steel Digital Story</t>
         </is>
       </c>
       <c r="G312" s="6" t="inlineStr">
         <is>
-          <t>Financial Express (CIO)</t>
+          <t>IFQM</t>
         </is>
       </c>
       <c r="H312" s="8" t="inlineStr"/>
       <c r="I312" s="9" t="inlineStr">
         <is>
-          <t>Tata Steel's iROC centre orchestrates 15+ steel plants globally using 250+ digital twin models.</t>
+          <t>Case study documenting Tata Steel's digital transformation journey including AI and digital twin deployment.</t>
         </is>
       </c>
       <c r="J312" s="10" t="inlineStr">
         <is>
-          <t>https://db.financialexpressb2b.com/features/how-tata-stee...</t>
+          <t>https://ifqm.org.in/product/tata-steel-digital-story/</t>
         </is>
       </c>
     </row>
@@ -15865,23 +15865,23 @@
       </c>
       <c r="F313" s="14" t="inlineStr">
         <is>
-          <t>Case Study: Tata Steel's AI Transformation</t>
+          <t>How Tata Steel has Transformed Plant And Mines With Digital Twins</t>
         </is>
       </c>
       <c r="G313" s="11" t="inlineStr">
         <is>
-          <t>AI Expert Network</t>
+          <t>Financial Express (CIO)</t>
         </is>
       </c>
       <c r="H313" s="13" t="inlineStr"/>
       <c r="I313" s="14" t="inlineStr">
         <is>
-          <t>Analysis of Tata Steel's AI transformation program covering sintering, blast furnace and thermal process optimization.</t>
+          <t>Tata Steel's iROC centre orchestrates 15+ steel plants globally using 250+ digital twin models.</t>
         </is>
       </c>
       <c r="J313" s="15" t="inlineStr">
         <is>
-          <t>https://aiexpert.network/case-study-tata-steels-ai-transf...</t>
+          <t>https://db.financialexpressb2b.com/features/how-tata-stee...</t>
         </is>
       </c>
     </row>
@@ -15913,23 +15913,23 @@
       </c>
       <c r="F314" s="9" t="inlineStr">
         <is>
-          <t>Digital Twins for Steel Plants: How Tata Steel Achieved $1.4 Billion in Savings</t>
+          <t>Case Study: Tata Steel's AI Transformation</t>
         </is>
       </c>
       <c r="G314" s="6" t="inlineStr">
         <is>
-          <t>iFactory (JRS Innovation)</t>
+          <t>AI Expert Network</t>
         </is>
       </c>
       <c r="H314" s="8" t="inlineStr"/>
       <c r="I314" s="9" t="inlineStr">
         <is>
-          <t>Tata Steel reported $1.4 billion cumulative cost savings five years after launching its digital twin transformation in 2015.</t>
+          <t>Analysis of Tata Steel's AI transformation program covering sintering, blast furnace and thermal process optimization.</t>
         </is>
       </c>
       <c r="J314" s="10" t="inlineStr">
         <is>
-          <t>https://ifactory.jrsinnovation.com/blog/tata-steel-digita...</t>
+          <t>https://aiexpert.network/case-study-tata-steels-ai-transf...</t>
         </is>
       </c>
     </row>
@@ -15946,34 +15946,38 @@
       </c>
       <c r="C315" s="12" t="inlineStr">
         <is>
-          <t>Tata Steel / JSW Steel / SAIL</t>
-        </is>
-      </c>
-      <c r="D315" s="13" t="inlineStr"/>
+          <t>Tata Steel</t>
+        </is>
+      </c>
+      <c r="D315" s="13" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
       <c r="E315" s="13" t="inlineStr">
         <is>
-          <t>Process/Yield</t>
+          <t>Digital twin</t>
         </is>
       </c>
       <c r="F315" s="14" t="inlineStr">
         <is>
-          <t>How AI Is Reforging India's Steel Industry</t>
+          <t>Digital Twins for Steel Plants: How Tata Steel Achieved $1.4 Billion in Savings</t>
         </is>
       </c>
       <c r="G315" s="11" t="inlineStr">
         <is>
-          <t>ARC Advisory Group</t>
+          <t>iFactory (JRS Innovation)</t>
         </is>
       </c>
       <c r="H315" s="13" t="inlineStr"/>
       <c r="I315" s="14" t="inlineStr">
         <is>
-          <t>Sector overview of AI adoption across Indian steelmakers including Tata Steel, JSW Steel and SAIL for efficiency gains.</t>
+          <t>Tata Steel reported $1.4 billion cumulative cost savings five years after launching its digital twin transformation in 2015.</t>
         </is>
       </c>
       <c r="J315" s="15" t="inlineStr">
         <is>
-          <t>https://www.arcweb.com/blog/how-ai-reforging-indias-steel...</t>
+          <t>https://ifactory.jrsinnovation.com/blog/tata-steel-digita...</t>
         </is>
       </c>
     </row>
@@ -18448,7 +18452,7 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
@@ -18598,14 +18602,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Energy &amp; Utilities</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>3</v>
-      </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
           <t>GenAI engineering</t>

</xml_diff>